<commit_message>
Add "Washed Potato Bag 4kg" via different-item flow
</commit_message>
<xml_diff>
--- a/shopping_list.xlsx
+++ b/shopping_list.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E1460"/>
+  <dimension ref="A1:E1462"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -25223,9 +25223,43 @@
         <v>2026-05-29</v>
       </c>
     </row>
+    <row r="1461">
+      <c r="A1461" t="str">
+        <v>Washed Potato Bag 4kg</v>
+      </c>
+      <c r="B1461">
+        <v>0</v>
+      </c>
+      <c r="C1461" t="str">
+        <v/>
+      </c>
+      <c r="D1461" t="str">
+        <v/>
+      </c>
+      <c r="E1461" t="str">
+        <v>2026-06-10</v>
+      </c>
+    </row>
+    <row r="1462">
+      <c r="A1462" t="str">
+        <v>Washed Potato Bag 4kg</v>
+      </c>
+      <c r="B1462">
+        <v>0</v>
+      </c>
+      <c r="C1462" t="str">
+        <v/>
+      </c>
+      <c r="D1462" t="str">
+        <v/>
+      </c>
+      <c r="E1462" t="str">
+        <v>2026-06-11</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E1460"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E1462"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>